<commit_message>
feat(provenance): porijeklo podataka i privola pružatelja — Excel, uvoz, claim, admin (Zadatak 17)
Predložak: 9 novih stupaca na kraj lista Pružatelji (izvor_podataka … google_place_id), padajuće liste, upute; regeneriran vendors-template.xlsx.
Backend: ProvenanceRules/ProvenanceMerge (parsiranje HR→interno, datumi UTC, prazno ne briše, refused→OptOut, uvoz nikad ne vraća OptOut,
privola preuzetog profila zaštićena), ConsentRules.GrantViaClaim (odobren claim = privola), ExcelImporter koristi, ReadSheet čita Excel datume kao ISO,
AdminController: GET/PUT /api/admin/vendors/{slug}/provenance + GET /api/admin/consent-summary.
Frontend: forma 'Porijeklo podataka i privola' + sažetak kampanje u /admin, lib/provenance.ts.
Testovi: ProvenanceTests (32), ClaimVerificationTests (+3).
Provjera: čista logika 91/91 + 7 mutacija; import-vendors.mjs daje identičan JSON s novim stupcima i bez njih; frontend tsc/build + browser;
importer/kontroleri/claim testovi nisu kompilirani (nema nuget).
</commit_message>
<xml_diff>
--- a/data/vendors-template.xlsx
+++ b/data/vendors-template.xlsx
@@ -310,6 +310,51 @@
     <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <t>Interno</t>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0" shapeId="0">
+      <text>
+        <t>Odakle su podaci o pružatelju: google_maps | web | instagram | facebook | partner | preporuka | drugo. INTERNO (GDPR evidencija — mnogi pružatelji su obrtnici, tj. fizičke osobe).</t>
+      </text>
+    </comment>
+    <comment ref="AB1" authorId="0" shapeId="0">
+      <text>
+        <t>Kad si prikupio podatke. Datum, npr. 30.09.2026. ili 2026-09-30.</t>
+      </text>
+    </comment>
+    <comment ref="AC1" authorId="0" shapeId="0">
+      <text>
+        <t>nepoznato | zatraženo | dano | odbijeno. 'odbijeno' = pružatelj ne želi biti na stranici → profil se automatski SKRIVA (opt-out). Preuzet profil (claim) se već vodi kao 'dano' i Excel ga ne smije vratiti na slabije.</t>
+      </text>
+    </comment>
+    <comment ref="AD1" authorId="0" shapeId="0">
+      <text>
+        <t>Kad si zatražio privolu (datum).</t>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="0" shapeId="0">
+      <text>
+        <t>Kad je pružatelj dao privolu (datum).</t>
+      </text>
+    </comment>
+    <comment ref="AF1" authorId="0" shapeId="0">
+      <text>
+        <t>Kako je privola zatražena/dana: email | instagram | facebook | telefon | osobno.</t>
+      </text>
+    </comment>
+    <comment ref="AG1" authorId="0" shapeId="0">
+      <text>
+        <t>Za što je privola dana, odvojeno zarezom: podaci, slike, recenzije.</t>
+      </text>
+    </comment>
+    <comment ref="AH1" authorId="0" shapeId="0">
+      <text>
+        <t>Interno — npr. 'pristao u DM-u 12.9., čeka potvrdu za slike'. U dnevniku promjena bilježi se samo 'promijenjeno', ne sadržaj.</t>
+      </text>
+    </comment>
+    <comment ref="AI1" authorId="0" shapeId="0">
+      <text>
+        <t>Google Place ID (npr. ChIJ…) — nađi ga preko Googleovog 'Place ID Finder'. SMIJE se spremati. NE kopiraj Google ocjene, recenzije ni fotografije (Googleovi uvjeti).</t>
       </text>
     </comment>
   </commentList>
@@ -635,7 +680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -837,12 +882,71 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>SAVJET ZA POČETAK:</t>
+          <t>PORIJEKLO PODATAKA I PRIVOLA (zadnjih 9 stupaca lista 'Pružatelji') — INTERNO, nikad javno:</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>• Mnogi pružatelji su obrtnici (fizičke osobe), pa evidentiramo odakle podaci i je li (i za što) pružatelj dao privolu. Sve su to POMOĆNI stupci — ostavi prazno ako ne znaš.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>• PRAZNA ĆELIJA NE BRIŠE: ako je stupac prazan, import ne dira vrijednost koja je već u bazi (admin je može ispraviti na stranici). Zato se ništa ne gubi ako Excel nema te podatke.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>• privola_status = 'odbijeno' → profil se pri uvozu automatski SKRIVA (opt-out). Import NIKAD ne vraća skriveni profil u prikaz — to radi samo admin (gumb 'Vrati u prikaz').</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>• Pružatelj koji preuzme profil (claim) automatski se vodi kao privola 'dano' (kanal claim); Excel to ne može vratiti na 'nepoznato' ni 'zatraženo'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>• google_place_id: Googleov 'Place ID Finder' (developers.google.com/maps/documentation/places/web-service/place-id) → pretraži poslovni naziv → kopiraj ID (počinje s ChIJ). Bez razmaka.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>• NE KOPIRAJ Google ocjene, broj recenzija, tekstove recenzija ni fotografije iz Googlea — Googleovi uvjeti to ne dopuštaju. Sprema se samo Place ID; živa ocjena se kasnije prikazuje izravno iz Googlea.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>• Datumi: 30.09.2026. ili 2026-09-30 (ili pravi Excel datum). Nepoznata vrijednost (npr. krivo napisan status) ispisuje se kao upozorenje i ignorira.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>SAVJET ZA POČETAK:</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>• Kreni s 1 regijom i 2–3 kategorije (npr. Dalmacija: Restorani i sale + Foto i Video) da provjeriš cijeli tok, pa širi.</t>
         </is>
@@ -859,7 +963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -878,6 +982,21 @@
           <t>Istraženo</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>nepoznato</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -895,6 +1014,21 @@
           <t>Kontaktirano</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>zatraženo</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -912,6 +1046,21 @@
           <t>Dozvola dobivena</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>dano</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -929,6 +1078,21 @@
           <t>Objavljeno</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>odbijeno</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>telefon</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -946,6 +1110,16 @@
           <t>Skriveno</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>partner</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>osobno</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -953,11 +1127,21 @@
           <t>Torte i kolači</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>preporuka</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
           <t>Foto i Video</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>drugo</t>
         </is>
       </c>
     </row>
@@ -1119,7 +1303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z6"/>
+  <dimension ref="A1:AI6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1148,6 +1332,15 @@
     <col width="22" customWidth="1" min="24" max="24"/>
     <col width="18" customWidth="1" min="25" max="25"/>
     <col width="30" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="16" customWidth="1" min="32" max="32"/>
+    <col width="22" customWidth="1" min="33" max="33"/>
+    <col width="30" customWidth="1" min="34" max="34"/>
+    <col width="28" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1281,6 +1474,51 @@
           <t>napomena</t>
         </is>
       </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>izvor_podataka</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>datum_prikupljanja</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>privola_status</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>privola_zatrazena</t>
+        </is>
+      </c>
+      <c r="AE1" s="3" t="inlineStr">
+        <is>
+          <t>privola_datum</t>
+        </is>
+      </c>
+      <c r="AF1" s="3" t="inlineStr">
+        <is>
+          <t>privola_kanal</t>
+        </is>
+      </c>
+      <c r="AG1" s="3" t="inlineStr">
+        <is>
+          <t>privola_opseg</t>
+        </is>
+      </c>
+      <c r="AH1" s="3" t="inlineStr">
+        <is>
+          <t>privola_napomena</t>
+        </is>
+      </c>
+      <c r="AI1" s="3" t="inlineStr">
+        <is>
+          <t>google_place_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -1393,6 +1631,51 @@
           <t>primjer — obriši ili ostavi (preskače se)</t>
         </is>
       </c>
+      <c r="AA2" s="4" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>30.09.2026.</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>dano</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>20.09.2026.</t>
+        </is>
+      </c>
+      <c r="AE2" s="4" t="inlineStr">
+        <is>
+          <t>29.09.2026.</t>
+        </is>
+      </c>
+      <c r="AF2" s="4" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="AG2" s="4" t="inlineStr">
+        <is>
+          <t>podaci, slike</t>
+        </is>
+      </c>
+      <c r="AH2" s="4" t="inlineStr">
+        <is>
+          <t>pristao mailom, slike uz navođenje autora</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
+        <is>
+          <t>ChIJ-primjer-place-id</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1499,6 +1782,39 @@
           <t>primjer — preskače se pri importu</t>
         </is>
       </c>
+      <c r="AA3" s="4" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="AB3" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="AC3" s="4" t="inlineStr">
+        <is>
+          <t>zatraženo</t>
+        </is>
+      </c>
+      <c r="AD3" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="AE3" s="4" t="inlineStr"/>
+      <c r="AF3" s="4" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="AG3" s="4" t="inlineStr"/>
+      <c r="AH3" s="4" t="inlineStr">
+        <is>
+          <t>poslan DM, čeka odgovor</t>
+        </is>
+      </c>
+      <c r="AI3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -1573,6 +1889,19 @@
           <t>primjer — bez grada/koordinata → bez pina</t>
         </is>
       </c>
+      <c r="AA4" s="4" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="AB4" s="4" t="inlineStr"/>
+      <c r="AC4" s="4" t="inlineStr"/>
+      <c r="AD4" s="4" t="inlineStr"/>
+      <c r="AE4" s="4" t="inlineStr"/>
+      <c r="AF4" s="4" t="inlineStr"/>
+      <c r="AG4" s="4" t="inlineStr"/>
+      <c r="AH4" s="4" t="inlineStr"/>
+      <c r="AI4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1641,6 +1970,23 @@
           <t>primjer — koordinate se geokodiraju iz grada</t>
         </is>
       </c>
+      <c r="AA5" s="4" t="inlineStr">
+        <is>
+          <t>preporuka</t>
+        </is>
+      </c>
+      <c r="AB5" s="4" t="inlineStr"/>
+      <c r="AC5" s="4" t="inlineStr">
+        <is>
+          <t>nepoznato</t>
+        </is>
+      </c>
+      <c r="AD5" s="4" t="inlineStr"/>
+      <c r="AE5" s="4" t="inlineStr"/>
+      <c r="AF5" s="4" t="inlineStr"/>
+      <c r="AG5" s="4" t="inlineStr"/>
+      <c r="AH5" s="4" t="inlineStr"/>
+      <c r="AI5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1745,9 +2091,38 @@
           <t>primjer — pokriva cijelu HR</t>
         </is>
       </c>
+      <c r="AA6" s="4" t="inlineStr">
+        <is>
+          <t>partner</t>
+        </is>
+      </c>
+      <c r="AB6" s="4" t="inlineStr"/>
+      <c r="AC6" s="4" t="inlineStr">
+        <is>
+          <t>dano</t>
+        </is>
+      </c>
+      <c r="AD6" s="4" t="inlineStr"/>
+      <c r="AE6" s="4" t="inlineStr">
+        <is>
+          <t>01.09.2026.</t>
+        </is>
+      </c>
+      <c r="AF6" s="4" t="inlineStr">
+        <is>
+          <t>osobno</t>
+        </is>
+      </c>
+      <c r="AG6" s="4" t="inlineStr">
+        <is>
+          <t>podaci, slike, recenzije</t>
+        </is>
+      </c>
+      <c r="AH6" s="4" t="inlineStr"/>
+      <c r="AI6" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="9">
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>Sifrarnici!$A$1:$A$28</formula1>
     </dataValidation>
@@ -1765,6 +2140,15 @@
     </dataValidation>
     <dataValidation sqref="Y2:Y500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Sifrarnici!$C$1:$C$5</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA2:AA500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>Sifrarnici!$D$1:$D$7</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC2:AC500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>Sifrarnici!$E$1:$E$4</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF2:AF500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>Sifrarnici!$F$1:$F$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>